<commit_message>
Affichage PDF intégré dans les exercices
</commit_message>
<xml_diff>
--- a/AVANCEMENT.xlsx
+++ b/AVANCEMENT.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/noemiejordi/Documents/_Ecole/03-Cycle3/MAT/01-Sequences/VLM/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A9E3A75-2A02-1F45-BEB9-81D534B86E42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4981BA43-8E2F-EA4F-B331-B46F57C96859}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" xr2:uid="{3DF85CC0-EEB2-D042-841B-46056AFB3A80}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="32">
   <si>
     <t>ex-008</t>
   </si>
@@ -123,6 +123,15 @@
   </si>
   <si>
     <t>ex-010</t>
+  </si>
+  <si>
+    <t>ex-011</t>
+  </si>
+  <si>
+    <t>ex-012</t>
+  </si>
+  <si>
+    <t>ex-013</t>
   </si>
 </sst>
 </file>
@@ -168,7 +177,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1">
@@ -179,6 +188,12 @@
       </extLst>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -530,21 +545,23 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B6C44A00-6051-A543-89C5-81FA429FBDD7}">
-  <dimension ref="A1:H170"/>
+  <dimension ref="A1:M170"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
-    <col min="1" max="1" width="16.5" style="1" customWidth="1"/>
+    <col min="1" max="1" width="8.5" style="5" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="30.6640625" style="1" customWidth="1"/>
     <col min="3" max="3" width="16" style="1" customWidth="1"/>
     <col min="4" max="4" width="12.83203125" style="1" customWidth="1"/>
     <col min="5" max="6" width="14.6640625" style="1" customWidth="1"/>
-    <col min="7" max="7" width="10.83203125" style="1"/>
-    <col min="8" max="8" width="54.1640625" style="1" customWidth="1"/>
-    <col min="9" max="16384" width="10.83203125" style="1"/>
+    <col min="7" max="7" width="54.1640625" style="1" customWidth="1"/>
+    <col min="8" max="8" width="10.83203125" style="1"/>
+    <col min="9" max="12" width="16" style="1" customWidth="1"/>
+    <col min="13" max="13" width="54.1640625" style="1" customWidth="1"/>
+    <col min="14" max="16384" width="10.83203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8">
-      <c r="A1" s="3" t="s">
+    <row r="1" spans="1:13">
+      <c r="A1" s="4" t="s">
         <v>7</v>
       </c>
       <c r="B1" s="3" t="s">
@@ -562,13 +579,27 @@
       <c r="F1" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="G1" s="3"/>
-      <c r="H1" s="3" t="s">
+      <c r="G1" s="3" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="2" spans="1:8">
-      <c r="A2" s="1">
+      <c r="I1" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="J1" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="K1" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="L1" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="M1" s="3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13">
+      <c r="A2" s="5">
         <v>1</v>
       </c>
       <c r="B2" s="3"/>
@@ -581,10 +612,21 @@
         <v>0</v>
       </c>
       <c r="G2" s="3"/>
-      <c r="H2" s="3"/>
-    </row>
-    <row r="3" spans="1:8">
-      <c r="A3" s="1">
+      <c r="I2" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="K2" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="L2" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13">
+      <c r="A3" s="5">
         <v>2</v>
       </c>
       <c r="B3" s="3"/>
@@ -597,10 +639,21 @@
         <v>0</v>
       </c>
       <c r="G3" s="3"/>
-      <c r="H3" s="3"/>
-    </row>
-    <row r="4" spans="1:8">
-      <c r="A4" s="1">
+      <c r="I3" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="J3" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="K3" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="L3" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13">
+      <c r="A4" s="5">
         <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
@@ -618,9 +671,21 @@
       <c r="F4" s="2" t="b">
         <v>0</v>
       </c>
-    </row>
-    <row r="5" spans="1:8">
-      <c r="A5" s="1">
+      <c r="I4" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="J4" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="K4" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="L4" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13">
+      <c r="A5" s="5">
         <v>4</v>
       </c>
       <c r="B5" s="1" t="s">
@@ -639,8 +704,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:8">
-      <c r="A6" s="1">
+    <row r="6" spans="1:13">
+      <c r="A6" s="5">
         <v>5</v>
       </c>
       <c r="B6" s="1" t="s">
@@ -659,8 +724,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:8">
-      <c r="A7" s="1">
+    <row r="7" spans="1:13">
+      <c r="A7" s="5">
         <v>6</v>
       </c>
       <c r="B7" s="1" t="s">
@@ -679,8 +744,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:8">
-      <c r="A8" s="1">
+    <row r="8" spans="1:13">
+      <c r="A8" s="5">
         <v>7</v>
       </c>
       <c r="B8" s="1" t="s">
@@ -699,8 +764,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:8">
-      <c r="A9" s="1">
+    <row r="9" spans="1:13">
+      <c r="A9" s="5">
         <v>8</v>
       </c>
       <c r="B9" s="1" t="s">
@@ -719,8 +784,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:8">
-      <c r="A10" s="1">
+    <row r="10" spans="1:13">
+      <c r="A10" s="5">
         <v>9</v>
       </c>
       <c r="B10" s="1" t="s">
@@ -739,8 +804,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:8">
-      <c r="A11" s="1">
+    <row r="11" spans="1:13">
+      <c r="A11" s="5">
         <v>10</v>
       </c>
       <c r="B11" s="1" t="s">
@@ -759,8 +824,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:8">
-      <c r="A12" s="1">
+    <row r="12" spans="1:13">
+      <c r="A12" s="5">
         <v>11</v>
       </c>
       <c r="B12" s="1" t="s">
@@ -773,14 +838,14 @@
         <v>6</v>
       </c>
       <c r="E12" s="2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F12" s="2" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:8">
-      <c r="A13" s="1">
+    <row r="13" spans="1:13">
+      <c r="A13" s="5">
         <v>12</v>
       </c>
       <c r="D13" s="1" t="s">
@@ -793,8 +858,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:8">
-      <c r="A14" s="1">
+    <row r="14" spans="1:13">
+      <c r="A14" s="5">
         <v>13</v>
       </c>
       <c r="D14" s="1" t="s">
@@ -807,8 +872,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:8">
-      <c r="A15" s="1">
+    <row r="15" spans="1:13">
+      <c r="A15" s="5">
         <v>14</v>
       </c>
       <c r="E15" s="2" t="b">
@@ -818,8 +883,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:8">
-      <c r="A16" s="1">
+    <row r="16" spans="1:13">
+      <c r="A16" s="5">
         <v>15</v>
       </c>
       <c r="E16" s="2" t="b">
@@ -830,7 +895,7 @@
       </c>
     </row>
     <row r="17" spans="1:6">
-      <c r="A17" s="1">
+      <c r="A17" s="5">
         <v>16</v>
       </c>
       <c r="E17" s="2" t="b">
@@ -841,7 +906,7 @@
       </c>
     </row>
     <row r="18" spans="1:6">
-      <c r="A18" s="1">
+      <c r="A18" s="5">
         <v>17</v>
       </c>
       <c r="E18" s="2" t="b">
@@ -852,7 +917,7 @@
       </c>
     </row>
     <row r="19" spans="1:6">
-      <c r="A19" s="1">
+      <c r="A19" s="5">
         <v>18</v>
       </c>
       <c r="E19" s="2" t="b">
@@ -863,7 +928,7 @@
       </c>
     </row>
     <row r="20" spans="1:6">
-      <c r="A20" s="1">
+      <c r="A20" s="5">
         <v>19</v>
       </c>
       <c r="B20" s="1" t="s">
@@ -883,7 +948,7 @@
       </c>
     </row>
     <row r="21" spans="1:6">
-      <c r="A21" s="1">
+      <c r="A21" s="5">
         <v>20</v>
       </c>
       <c r="E21" s="2" t="b">
@@ -894,7 +959,7 @@
       </c>
     </row>
     <row r="22" spans="1:6">
-      <c r="A22" s="1">
+      <c r="A22" s="5">
         <v>21</v>
       </c>
       <c r="E22" s="2" t="b">
@@ -905,7 +970,7 @@
       </c>
     </row>
     <row r="23" spans="1:6">
-      <c r="A23" s="1">
+      <c r="A23" s="5">
         <v>22</v>
       </c>
       <c r="E23" s="2" t="b">
@@ -916,7 +981,7 @@
       </c>
     </row>
     <row r="24" spans="1:6">
-      <c r="A24" s="1">
+      <c r="A24" s="5">
         <v>23</v>
       </c>
       <c r="E24" s="2" t="b">
@@ -927,7 +992,7 @@
       </c>
     </row>
     <row r="25" spans="1:6">
-      <c r="A25" s="1">
+      <c r="A25" s="5">
         <v>24</v>
       </c>
       <c r="E25" s="2" t="b">
@@ -938,7 +1003,7 @@
       </c>
     </row>
     <row r="26" spans="1:6">
-      <c r="A26" s="1">
+      <c r="A26" s="5">
         <v>25</v>
       </c>
       <c r="E26" s="2" t="b">
@@ -949,7 +1014,7 @@
       </c>
     </row>
     <row r="27" spans="1:6">
-      <c r="A27" s="1">
+      <c r="A27" s="5">
         <v>26</v>
       </c>
       <c r="E27" s="2" t="b">
@@ -960,7 +1025,7 @@
       </c>
     </row>
     <row r="28" spans="1:6">
-      <c r="A28" s="1">
+      <c r="A28" s="5">
         <v>27</v>
       </c>
       <c r="E28" s="2" t="b">
@@ -971,7 +1036,7 @@
       </c>
     </row>
     <row r="29" spans="1:6">
-      <c r="A29" s="1">
+      <c r="A29" s="5">
         <v>28</v>
       </c>
       <c r="E29" s="2" t="b">
@@ -982,7 +1047,7 @@
       </c>
     </row>
     <row r="30" spans="1:6">
-      <c r="A30" s="1">
+      <c r="A30" s="5">
         <v>29</v>
       </c>
       <c r="E30" s="2" t="b">
@@ -993,7 +1058,7 @@
       </c>
     </row>
     <row r="31" spans="1:6">
-      <c r="A31" s="1">
+      <c r="A31" s="5">
         <v>30</v>
       </c>
       <c r="E31" s="2" t="b">
@@ -1004,7 +1069,7 @@
       </c>
     </row>
     <row r="32" spans="1:6">
-      <c r="A32" s="1">
+      <c r="A32" s="5">
         <v>31</v>
       </c>
       <c r="E32" s="2" t="b">
@@ -1015,7 +1080,7 @@
       </c>
     </row>
     <row r="33" spans="1:6">
-      <c r="A33" s="1">
+      <c r="A33" s="5">
         <v>32</v>
       </c>
       <c r="E33" s="2" t="b">
@@ -1026,7 +1091,7 @@
       </c>
     </row>
     <row r="34" spans="1:6">
-      <c r="A34" s="1">
+      <c r="A34" s="5">
         <v>33</v>
       </c>
       <c r="E34" s="2" t="b">
@@ -1037,7 +1102,7 @@
       </c>
     </row>
     <row r="35" spans="1:6">
-      <c r="A35" s="1">
+      <c r="A35" s="5">
         <v>34</v>
       </c>
       <c r="E35" s="2" t="b">
@@ -1048,7 +1113,7 @@
       </c>
     </row>
     <row r="36" spans="1:6">
-      <c r="A36" s="1">
+      <c r="A36" s="5">
         <v>35</v>
       </c>
       <c r="E36" s="2" t="b">
@@ -1059,7 +1124,7 @@
       </c>
     </row>
     <row r="37" spans="1:6">
-      <c r="A37" s="1">
+      <c r="A37" s="5">
         <v>36</v>
       </c>
       <c r="E37" s="2" t="b">
@@ -1070,7 +1135,7 @@
       </c>
     </row>
     <row r="38" spans="1:6">
-      <c r="A38" s="1">
+      <c r="A38" s="5">
         <v>37</v>
       </c>
       <c r="E38" s="2" t="b">
@@ -1081,7 +1146,7 @@
       </c>
     </row>
     <row r="39" spans="1:6">
-      <c r="A39" s="1">
+      <c r="A39" s="5">
         <v>38</v>
       </c>
       <c r="E39" s="2" t="b">
@@ -1092,7 +1157,7 @@
       </c>
     </row>
     <row r="40" spans="1:6">
-      <c r="A40" s="1">
+      <c r="A40" s="5">
         <v>39</v>
       </c>
       <c r="E40" s="2" t="b">
@@ -1103,7 +1168,7 @@
       </c>
     </row>
     <row r="41" spans="1:6">
-      <c r="A41" s="1">
+      <c r="A41" s="5">
         <v>40</v>
       </c>
       <c r="E41" s="2" t="b">
@@ -1114,7 +1179,7 @@
       </c>
     </row>
     <row r="42" spans="1:6">
-      <c r="A42" s="1">
+      <c r="A42" s="5">
         <v>41</v>
       </c>
       <c r="E42" s="2" t="b">
@@ -1125,7 +1190,7 @@
       </c>
     </row>
     <row r="43" spans="1:6">
-      <c r="A43" s="1">
+      <c r="A43" s="5">
         <v>42</v>
       </c>
       <c r="E43" s="2" t="b">
@@ -1136,7 +1201,7 @@
       </c>
     </row>
     <row r="44" spans="1:6">
-      <c r="A44" s="1">
+      <c r="A44" s="5">
         <v>43</v>
       </c>
       <c r="E44" s="2" t="b">
@@ -1147,7 +1212,7 @@
       </c>
     </row>
     <row r="45" spans="1:6">
-      <c r="A45" s="1">
+      <c r="A45" s="5">
         <v>44</v>
       </c>
       <c r="E45" s="2" t="b">
@@ -1158,7 +1223,7 @@
       </c>
     </row>
     <row r="46" spans="1:6">
-      <c r="A46" s="1">
+      <c r="A46" s="5">
         <v>45</v>
       </c>
       <c r="E46" s="2" t="b">
@@ -1169,7 +1234,7 @@
       </c>
     </row>
     <row r="47" spans="1:6">
-      <c r="A47" s="1">
+      <c r="A47" s="5">
         <v>46</v>
       </c>
       <c r="E47" s="2" t="b">
@@ -1180,7 +1245,7 @@
       </c>
     </row>
     <row r="48" spans="1:6">
-      <c r="A48" s="1">
+      <c r="A48" s="5">
         <v>47</v>
       </c>
       <c r="E48" s="2" t="b">
@@ -1191,7 +1256,7 @@
       </c>
     </row>
     <row r="49" spans="1:6">
-      <c r="A49" s="1">
+      <c r="A49" s="5">
         <v>48</v>
       </c>
       <c r="E49" s="2" t="b">
@@ -1202,7 +1267,7 @@
       </c>
     </row>
     <row r="50" spans="1:6">
-      <c r="A50" s="1">
+      <c r="A50" s="5">
         <v>49</v>
       </c>
       <c r="E50" s="2" t="b">
@@ -1213,7 +1278,7 @@
       </c>
     </row>
     <row r="51" spans="1:6">
-      <c r="A51" s="1">
+      <c r="A51" s="5">
         <v>50</v>
       </c>
       <c r="E51" s="2" t="b">
@@ -1224,7 +1289,7 @@
       </c>
     </row>
     <row r="52" spans="1:6">
-      <c r="A52" s="1">
+      <c r="A52" s="5">
         <v>51</v>
       </c>
       <c r="E52" s="2" t="b">
@@ -1235,7 +1300,7 @@
       </c>
     </row>
     <row r="53" spans="1:6">
-      <c r="A53" s="1">
+      <c r="A53" s="5">
         <v>52</v>
       </c>
       <c r="E53" s="2" t="b">
@@ -1246,7 +1311,7 @@
       </c>
     </row>
     <row r="54" spans="1:6">
-      <c r="A54" s="1">
+      <c r="A54" s="5">
         <v>53</v>
       </c>
       <c r="E54" s="2" t="b">
@@ -1257,7 +1322,7 @@
       </c>
     </row>
     <row r="55" spans="1:6">
-      <c r="A55" s="1">
+      <c r="A55" s="5">
         <v>54</v>
       </c>
       <c r="E55" s="2" t="b">
@@ -1268,7 +1333,7 @@
       </c>
     </row>
     <row r="56" spans="1:6">
-      <c r="A56" s="1">
+      <c r="A56" s="5">
         <v>55</v>
       </c>
       <c r="E56" s="2" t="b">
@@ -1279,7 +1344,7 @@
       </c>
     </row>
     <row r="57" spans="1:6">
-      <c r="A57" s="1">
+      <c r="A57" s="5">
         <v>56</v>
       </c>
       <c r="E57" s="2" t="b">
@@ -1290,7 +1355,7 @@
       </c>
     </row>
     <row r="58" spans="1:6">
-      <c r="A58" s="1">
+      <c r="A58" s="5">
         <v>57</v>
       </c>
       <c r="E58" s="2" t="b">
@@ -1301,7 +1366,7 @@
       </c>
     </row>
     <row r="59" spans="1:6">
-      <c r="A59" s="1">
+      <c r="A59" s="5">
         <v>58</v>
       </c>
       <c r="E59" s="2" t="b">
@@ -1312,7 +1377,7 @@
       </c>
     </row>
     <row r="60" spans="1:6">
-      <c r="A60" s="1">
+      <c r="A60" s="5">
         <v>59</v>
       </c>
       <c r="E60" s="2" t="b">
@@ -1323,7 +1388,7 @@
       </c>
     </row>
     <row r="61" spans="1:6">
-      <c r="A61" s="1">
+      <c r="A61" s="5">
         <v>60</v>
       </c>
       <c r="E61" s="2" t="b">
@@ -1334,7 +1399,7 @@
       </c>
     </row>
     <row r="62" spans="1:6">
-      <c r="A62" s="1">
+      <c r="A62" s="5">
         <v>61</v>
       </c>
       <c r="E62" s="2" t="b">
@@ -1345,7 +1410,7 @@
       </c>
     </row>
     <row r="63" spans="1:6">
-      <c r="A63" s="1">
+      <c r="A63" s="5">
         <v>62</v>
       </c>
       <c r="E63" s="2" t="b">
@@ -1356,7 +1421,7 @@
       </c>
     </row>
     <row r="64" spans="1:6">
-      <c r="A64" s="1">
+      <c r="A64" s="5">
         <v>63</v>
       </c>
       <c r="E64" s="2" t="b">
@@ -1367,7 +1432,7 @@
       </c>
     </row>
     <row r="65" spans="1:6">
-      <c r="A65" s="1">
+      <c r="A65" s="5">
         <v>64</v>
       </c>
       <c r="E65" s="2" t="b">
@@ -1378,7 +1443,7 @@
       </c>
     </row>
     <row r="66" spans="1:6">
-      <c r="A66" s="1">
+      <c r="A66" s="5">
         <v>65</v>
       </c>
       <c r="E66" s="2" t="b">
@@ -1389,7 +1454,7 @@
       </c>
     </row>
     <row r="67" spans="1:6">
-      <c r="A67" s="1">
+      <c r="A67" s="5">
         <v>66</v>
       </c>
       <c r="E67" s="2" t="b">
@@ -1400,7 +1465,7 @@
       </c>
     </row>
     <row r="68" spans="1:6">
-      <c r="A68" s="1">
+      <c r="A68" s="5">
         <v>67</v>
       </c>
       <c r="E68" s="2" t="b">
@@ -1411,7 +1476,7 @@
       </c>
     </row>
     <row r="69" spans="1:6">
-      <c r="A69" s="1">
+      <c r="A69" s="5">
         <v>68</v>
       </c>
       <c r="E69" s="2" t="b">
@@ -1422,7 +1487,7 @@
       </c>
     </row>
     <row r="70" spans="1:6">
-      <c r="A70" s="1">
+      <c r="A70" s="5">
         <v>69</v>
       </c>
       <c r="E70" s="2" t="b">
@@ -1433,7 +1498,7 @@
       </c>
     </row>
     <row r="71" spans="1:6">
-      <c r="A71" s="1">
+      <c r="A71" s="5">
         <v>70</v>
       </c>
       <c r="E71" s="2" t="b">
@@ -1444,7 +1509,7 @@
       </c>
     </row>
     <row r="72" spans="1:6">
-      <c r="A72" s="1">
+      <c r="A72" s="5">
         <v>71</v>
       </c>
       <c r="E72" s="2" t="b">
@@ -1455,7 +1520,7 @@
       </c>
     </row>
     <row r="73" spans="1:6">
-      <c r="A73" s="1">
+      <c r="A73" s="5">
         <v>72</v>
       </c>
       <c r="E73" s="2" t="b">
@@ -1466,7 +1531,7 @@
       </c>
     </row>
     <row r="74" spans="1:6">
-      <c r="A74" s="1">
+      <c r="A74" s="5">
         <v>73</v>
       </c>
       <c r="E74" s="2" t="b">
@@ -1477,7 +1542,7 @@
       </c>
     </row>
     <row r="75" spans="1:6">
-      <c r="A75" s="1">
+      <c r="A75" s="5">
         <v>74</v>
       </c>
       <c r="E75" s="2" t="b">
@@ -1488,7 +1553,7 @@
       </c>
     </row>
     <row r="76" spans="1:6">
-      <c r="A76" s="1">
+      <c r="A76" s="5">
         <v>75</v>
       </c>
       <c r="E76" s="2" t="b">
@@ -1499,7 +1564,7 @@
       </c>
     </row>
     <row r="77" spans="1:6">
-      <c r="A77" s="1">
+      <c r="A77" s="5">
         <v>76</v>
       </c>
       <c r="E77" s="2" t="b">
@@ -1510,7 +1575,7 @@
       </c>
     </row>
     <row r="78" spans="1:6">
-      <c r="A78" s="1">
+      <c r="A78" s="5">
         <v>77</v>
       </c>
       <c r="E78" s="2" t="b">
@@ -1521,7 +1586,7 @@
       </c>
     </row>
     <row r="79" spans="1:6">
-      <c r="A79" s="1">
+      <c r="A79" s="5">
         <v>78</v>
       </c>
       <c r="E79" s="2" t="b">
@@ -1532,7 +1597,7 @@
       </c>
     </row>
     <row r="80" spans="1:6">
-      <c r="A80" s="1">
+      <c r="A80" s="5">
         <v>79</v>
       </c>
       <c r="E80" s="2" t="b">
@@ -1543,7 +1608,7 @@
       </c>
     </row>
     <row r="81" spans="1:6">
-      <c r="A81" s="1">
+      <c r="A81" s="5">
         <v>80</v>
       </c>
       <c r="E81" s="2" t="b">
@@ -1554,7 +1619,7 @@
       </c>
     </row>
     <row r="82" spans="1:6">
-      <c r="A82" s="1">
+      <c r="A82" s="5">
         <v>81</v>
       </c>
       <c r="E82" s="2" t="b">
@@ -1565,7 +1630,7 @@
       </c>
     </row>
     <row r="83" spans="1:6">
-      <c r="A83" s="1">
+      <c r="A83" s="5">
         <v>82</v>
       </c>
       <c r="E83" s="2" t="b">
@@ -1576,7 +1641,7 @@
       </c>
     </row>
     <row r="84" spans="1:6">
-      <c r="A84" s="1">
+      <c r="A84" s="5">
         <v>83</v>
       </c>
       <c r="E84" s="2" t="b">
@@ -1587,7 +1652,7 @@
       </c>
     </row>
     <row r="85" spans="1:6">
-      <c r="A85" s="1">
+      <c r="A85" s="5">
         <v>84</v>
       </c>
       <c r="E85" s="2" t="b">
@@ -1598,7 +1663,7 @@
       </c>
     </row>
     <row r="86" spans="1:6">
-      <c r="A86" s="1">
+      <c r="A86" s="5">
         <v>85</v>
       </c>
       <c r="E86" s="2" t="b">
@@ -1609,7 +1674,7 @@
       </c>
     </row>
     <row r="87" spans="1:6">
-      <c r="A87" s="1">
+      <c r="A87" s="5">
         <v>86</v>
       </c>
       <c r="E87" s="2" t="b">
@@ -1620,7 +1685,7 @@
       </c>
     </row>
     <row r="88" spans="1:6">
-      <c r="A88" s="1">
+      <c r="A88" s="5">
         <v>87</v>
       </c>
       <c r="E88" s="2" t="b">
@@ -1631,7 +1696,7 @@
       </c>
     </row>
     <row r="89" spans="1:6">
-      <c r="A89" s="1">
+      <c r="A89" s="5">
         <v>88</v>
       </c>
       <c r="E89" s="2" t="b">
@@ -1642,7 +1707,7 @@
       </c>
     </row>
     <row r="90" spans="1:6">
-      <c r="A90" s="1">
+      <c r="A90" s="5">
         <v>89</v>
       </c>
       <c r="E90" s="2" t="b">
@@ -1653,7 +1718,7 @@
       </c>
     </row>
     <row r="91" spans="1:6">
-      <c r="A91" s="1">
+      <c r="A91" s="5">
         <v>90</v>
       </c>
       <c r="E91" s="2" t="b">
@@ -1664,7 +1729,7 @@
       </c>
     </row>
     <row r="92" spans="1:6">
-      <c r="A92" s="1">
+      <c r="A92" s="5">
         <v>91</v>
       </c>
       <c r="E92" s="2" t="b">
@@ -1675,7 +1740,7 @@
       </c>
     </row>
     <row r="93" spans="1:6">
-      <c r="A93" s="1">
+      <c r="A93" s="5">
         <v>92</v>
       </c>
       <c r="E93" s="2" t="b">
@@ -1686,7 +1751,7 @@
       </c>
     </row>
     <row r="94" spans="1:6">
-      <c r="A94" s="1">
+      <c r="A94" s="5">
         <v>93</v>
       </c>
       <c r="E94" s="2" t="b">
@@ -1697,7 +1762,7 @@
       </c>
     </row>
     <row r="95" spans="1:6">
-      <c r="A95" s="1">
+      <c r="A95" s="5">
         <v>94</v>
       </c>
       <c r="E95" s="2" t="b">
@@ -1708,7 +1773,7 @@
       </c>
     </row>
     <row r="96" spans="1:6">
-      <c r="A96" s="1">
+      <c r="A96" s="5">
         <v>95</v>
       </c>
       <c r="E96" s="2" t="b">
@@ -1719,7 +1784,7 @@
       </c>
     </row>
     <row r="97" spans="1:6">
-      <c r="A97" s="1">
+      <c r="A97" s="5">
         <v>96</v>
       </c>
       <c r="E97" s="2" t="b">
@@ -1730,7 +1795,7 @@
       </c>
     </row>
     <row r="98" spans="1:6">
-      <c r="A98" s="1">
+      <c r="A98" s="5">
         <v>97</v>
       </c>
       <c r="E98" s="2" t="b">
@@ -1741,7 +1806,7 @@
       </c>
     </row>
     <row r="99" spans="1:6">
-      <c r="A99" s="1">
+      <c r="A99" s="5">
         <v>98</v>
       </c>
       <c r="E99" s="2" t="b">
@@ -1752,7 +1817,7 @@
       </c>
     </row>
     <row r="100" spans="1:6">
-      <c r="A100" s="1">
+      <c r="A100" s="5">
         <v>99</v>
       </c>
       <c r="E100" s="2" t="b">
@@ -1763,7 +1828,7 @@
       </c>
     </row>
     <row r="101" spans="1:6">
-      <c r="A101" s="1">
+      <c r="A101" s="5">
         <v>100</v>
       </c>
       <c r="E101" s="2" t="b">
@@ -1774,7 +1839,7 @@
       </c>
     </row>
     <row r="102" spans="1:6">
-      <c r="A102" s="1">
+      <c r="A102" s="5">
         <v>101</v>
       </c>
       <c r="E102" s="2" t="b">
@@ -1785,7 +1850,7 @@
       </c>
     </row>
     <row r="103" spans="1:6">
-      <c r="A103" s="1">
+      <c r="A103" s="5">
         <v>102</v>
       </c>
       <c r="E103" s="2" t="b">
@@ -1796,7 +1861,7 @@
       </c>
     </row>
     <row r="104" spans="1:6">
-      <c r="A104" s="1">
+      <c r="A104" s="5">
         <v>103</v>
       </c>
       <c r="E104" s="2" t="b">
@@ -1807,7 +1872,7 @@
       </c>
     </row>
     <row r="105" spans="1:6">
-      <c r="A105" s="1">
+      <c r="A105" s="5">
         <v>104</v>
       </c>
       <c r="E105" s="2" t="b">
@@ -1818,7 +1883,7 @@
       </c>
     </row>
     <row r="106" spans="1:6">
-      <c r="A106" s="1">
+      <c r="A106" s="5">
         <v>105</v>
       </c>
       <c r="E106" s="2" t="b">
@@ -1829,7 +1894,7 @@
       </c>
     </row>
     <row r="107" spans="1:6">
-      <c r="A107" s="1">
+      <c r="A107" s="5">
         <v>106</v>
       </c>
       <c r="E107" s="2" t="b">
@@ -1840,7 +1905,7 @@
       </c>
     </row>
     <row r="108" spans="1:6">
-      <c r="A108" s="1">
+      <c r="A108" s="5">
         <v>107</v>
       </c>
       <c r="E108" s="2" t="b">
@@ -1851,7 +1916,7 @@
       </c>
     </row>
     <row r="109" spans="1:6">
-      <c r="A109" s="1">
+      <c r="A109" s="5">
         <v>108</v>
       </c>
       <c r="E109" s="2" t="b">
@@ -1862,7 +1927,7 @@
       </c>
     </row>
     <row r="110" spans="1:6">
-      <c r="A110" s="1">
+      <c r="A110" s="5">
         <v>109</v>
       </c>
       <c r="E110" s="2" t="b">
@@ -1873,7 +1938,7 @@
       </c>
     </row>
     <row r="111" spans="1:6">
-      <c r="A111" s="1">
+      <c r="A111" s="5">
         <v>110</v>
       </c>
       <c r="E111" s="2" t="b">
@@ -1884,7 +1949,7 @@
       </c>
     </row>
     <row r="112" spans="1:6">
-      <c r="A112" s="1">
+      <c r="A112" s="5">
         <v>111</v>
       </c>
       <c r="E112" s="2" t="b">
@@ -1895,7 +1960,7 @@
       </c>
     </row>
     <row r="113" spans="1:6">
-      <c r="A113" s="1">
+      <c r="A113" s="5">
         <v>112</v>
       </c>
       <c r="E113" s="2" t="b">
@@ -1906,7 +1971,7 @@
       </c>
     </row>
     <row r="114" spans="1:6">
-      <c r="A114" s="1">
+      <c r="A114" s="5">
         <v>113</v>
       </c>
       <c r="E114" s="2" t="b">
@@ -1917,7 +1982,7 @@
       </c>
     </row>
     <row r="115" spans="1:6">
-      <c r="A115" s="1">
+      <c r="A115" s="5">
         <v>114</v>
       </c>
       <c r="E115" s="2" t="b">
@@ -1928,7 +1993,7 @@
       </c>
     </row>
     <row r="116" spans="1:6">
-      <c r="A116" s="1">
+      <c r="A116" s="5">
         <v>115</v>
       </c>
       <c r="E116" s="2" t="b">
@@ -1939,7 +2004,7 @@
       </c>
     </row>
     <row r="117" spans="1:6">
-      <c r="A117" s="1">
+      <c r="A117" s="5">
         <v>116</v>
       </c>
       <c r="E117" s="2" t="b">
@@ -1950,7 +2015,7 @@
       </c>
     </row>
     <row r="118" spans="1:6">
-      <c r="A118" s="1">
+      <c r="A118" s="5">
         <v>117</v>
       </c>
       <c r="E118" s="2" t="b">
@@ -1961,7 +2026,7 @@
       </c>
     </row>
     <row r="119" spans="1:6">
-      <c r="A119" s="1">
+      <c r="A119" s="5">
         <v>118</v>
       </c>
       <c r="E119" s="2" t="b">
@@ -1972,7 +2037,7 @@
       </c>
     </row>
     <row r="120" spans="1:6">
-      <c r="A120" s="1">
+      <c r="A120" s="5">
         <v>119</v>
       </c>
       <c r="E120" s="2" t="b">
@@ -1983,7 +2048,7 @@
       </c>
     </row>
     <row r="121" spans="1:6">
-      <c r="A121" s="1">
+      <c r="A121" s="5">
         <v>120</v>
       </c>
       <c r="E121" s="2" t="b">
@@ -1994,7 +2059,7 @@
       </c>
     </row>
     <row r="122" spans="1:6">
-      <c r="A122" s="1">
+      <c r="A122" s="5">
         <v>121</v>
       </c>
       <c r="E122" s="2" t="b">
@@ -2005,7 +2070,7 @@
       </c>
     </row>
     <row r="123" spans="1:6">
-      <c r="A123" s="1">
+      <c r="A123" s="5">
         <v>122</v>
       </c>
       <c r="E123" s="2" t="b">
@@ -2016,7 +2081,7 @@
       </c>
     </row>
     <row r="124" spans="1:6">
-      <c r="A124" s="1">
+      <c r="A124" s="5">
         <v>123</v>
       </c>
       <c r="E124" s="2" t="b">
@@ -2027,7 +2092,7 @@
       </c>
     </row>
     <row r="125" spans="1:6">
-      <c r="A125" s="1">
+      <c r="A125" s="5">
         <v>124</v>
       </c>
       <c r="E125" s="2" t="b">
@@ -2038,7 +2103,7 @@
       </c>
     </row>
     <row r="126" spans="1:6">
-      <c r="A126" s="1">
+      <c r="A126" s="5">
         <v>125</v>
       </c>
       <c r="E126" s="2" t="b">
@@ -2049,7 +2114,7 @@
       </c>
     </row>
     <row r="127" spans="1:6">
-      <c r="A127" s="1">
+      <c r="A127" s="5">
         <v>126</v>
       </c>
       <c r="E127" s="2" t="b">
@@ -2060,7 +2125,7 @@
       </c>
     </row>
     <row r="128" spans="1:6">
-      <c r="A128" s="1">
+      <c r="A128" s="5">
         <v>127</v>
       </c>
       <c r="E128" s="2" t="b">
@@ -2071,7 +2136,7 @@
       </c>
     </row>
     <row r="129" spans="1:6">
-      <c r="A129" s="1">
+      <c r="A129" s="5">
         <v>128</v>
       </c>
       <c r="E129" s="2" t="b">
@@ -2082,7 +2147,7 @@
       </c>
     </row>
     <row r="130" spans="1:6">
-      <c r="A130" s="1">
+      <c r="A130" s="5">
         <v>129</v>
       </c>
       <c r="E130" s="2" t="b">
@@ -2093,7 +2158,7 @@
       </c>
     </row>
     <row r="131" spans="1:6">
-      <c r="A131" s="1">
+      <c r="A131" s="5">
         <v>130</v>
       </c>
       <c r="E131" s="2" t="b">
@@ -2104,7 +2169,7 @@
       </c>
     </row>
     <row r="132" spans="1:6">
-      <c r="A132" s="1">
+      <c r="A132" s="5">
         <v>131</v>
       </c>
       <c r="E132" s="2" t="b">
@@ -2115,7 +2180,7 @@
       </c>
     </row>
     <row r="133" spans="1:6">
-      <c r="A133" s="1">
+      <c r="A133" s="5">
         <v>132</v>
       </c>
       <c r="E133" s="2" t="b">
@@ -2126,7 +2191,7 @@
       </c>
     </row>
     <row r="134" spans="1:6">
-      <c r="A134" s="1">
+      <c r="A134" s="5">
         <v>133</v>
       </c>
       <c r="E134" s="2" t="b">
@@ -2137,7 +2202,7 @@
       </c>
     </row>
     <row r="135" spans="1:6">
-      <c r="A135" s="1">
+      <c r="A135" s="5">
         <v>134</v>
       </c>
       <c r="E135" s="2" t="b">
@@ -2148,7 +2213,7 @@
       </c>
     </row>
     <row r="136" spans="1:6">
-      <c r="A136" s="1">
+      <c r="A136" s="5">
         <v>135</v>
       </c>
       <c r="E136" s="2" t="b">
@@ -2159,7 +2224,7 @@
       </c>
     </row>
     <row r="137" spans="1:6">
-      <c r="A137" s="1">
+      <c r="A137" s="5">
         <v>136</v>
       </c>
       <c r="E137" s="2" t="b">
@@ -2170,7 +2235,7 @@
       </c>
     </row>
     <row r="138" spans="1:6">
-      <c r="A138" s="1">
+      <c r="A138" s="5">
         <v>137</v>
       </c>
       <c r="E138" s="2" t="b">
@@ -2181,7 +2246,7 @@
       </c>
     </row>
     <row r="139" spans="1:6">
-      <c r="A139" s="1">
+      <c r="A139" s="5">
         <v>138</v>
       </c>
       <c r="E139" s="2" t="b">
@@ -2192,7 +2257,7 @@
       </c>
     </row>
     <row r="140" spans="1:6">
-      <c r="A140" s="1">
+      <c r="A140" s="5">
         <v>139</v>
       </c>
       <c r="E140" s="2" t="b">
@@ -2203,7 +2268,7 @@
       </c>
     </row>
     <row r="141" spans="1:6">
-      <c r="A141" s="1">
+      <c r="A141" s="5">
         <v>140</v>
       </c>
       <c r="E141" s="2" t="b">
@@ -2214,7 +2279,7 @@
       </c>
     </row>
     <row r="142" spans="1:6">
-      <c r="A142" s="1">
+      <c r="A142" s="5">
         <v>141</v>
       </c>
       <c r="E142" s="2" t="b">
@@ -2225,7 +2290,7 @@
       </c>
     </row>
     <row r="143" spans="1:6">
-      <c r="A143" s="1">
+      <c r="A143" s="5">
         <v>142</v>
       </c>
       <c r="E143" s="2" t="b">
@@ -2236,7 +2301,7 @@
       </c>
     </row>
     <row r="144" spans="1:6">
-      <c r="A144" s="1">
+      <c r="A144" s="5">
         <v>143</v>
       </c>
       <c r="E144" s="2" t="b">
@@ -2247,7 +2312,7 @@
       </c>
     </row>
     <row r="145" spans="1:6">
-      <c r="A145" s="1">
+      <c r="A145" s="5">
         <v>144</v>
       </c>
       <c r="E145" s="2" t="b">
@@ -2258,7 +2323,7 @@
       </c>
     </row>
     <row r="146" spans="1:6">
-      <c r="A146" s="1">
+      <c r="A146" s="5">
         <v>145</v>
       </c>
       <c r="E146" s="2" t="b">
@@ -2269,7 +2334,7 @@
       </c>
     </row>
     <row r="147" spans="1:6">
-      <c r="A147" s="1">
+      <c r="A147" s="5">
         <v>146</v>
       </c>
       <c r="E147" s="2" t="b">
@@ -2280,7 +2345,7 @@
       </c>
     </row>
     <row r="148" spans="1:6">
-      <c r="A148" s="1">
+      <c r="A148" s="5">
         <v>147</v>
       </c>
       <c r="E148" s="2" t="b">
@@ -2291,7 +2356,7 @@
       </c>
     </row>
     <row r="149" spans="1:6">
-      <c r="A149" s="1">
+      <c r="A149" s="5">
         <v>148</v>
       </c>
       <c r="E149" s="2" t="b">
@@ -2302,7 +2367,7 @@
       </c>
     </row>
     <row r="150" spans="1:6">
-      <c r="A150" s="1">
+      <c r="A150" s="5">
         <v>149</v>
       </c>
       <c r="E150" s="2" t="b">
@@ -2313,7 +2378,7 @@
       </c>
     </row>
     <row r="151" spans="1:6">
-      <c r="A151" s="1">
+      <c r="A151" s="5">
         <v>150</v>
       </c>
       <c r="E151" s="2" t="b">
@@ -2324,7 +2389,7 @@
       </c>
     </row>
     <row r="152" spans="1:6">
-      <c r="A152" s="1">
+      <c r="A152" s="5">
         <v>151</v>
       </c>
       <c r="E152" s="2" t="b">
@@ -2335,7 +2400,7 @@
       </c>
     </row>
     <row r="153" spans="1:6">
-      <c r="A153" s="1">
+      <c r="A153" s="5">
         <v>152</v>
       </c>
       <c r="E153" s="2" t="b">
@@ -2346,7 +2411,7 @@
       </c>
     </row>
     <row r="154" spans="1:6">
-      <c r="A154" s="1">
+      <c r="A154" s="5">
         <v>153</v>
       </c>
       <c r="E154" s="2" t="b">
@@ -2357,7 +2422,7 @@
       </c>
     </row>
     <row r="155" spans="1:6">
-      <c r="A155" s="1">
+      <c r="A155" s="5">
         <v>154</v>
       </c>
       <c r="E155" s="2" t="b">
@@ -2368,7 +2433,7 @@
       </c>
     </row>
     <row r="156" spans="1:6">
-      <c r="A156" s="1">
+      <c r="A156" s="5">
         <v>155</v>
       </c>
       <c r="E156" s="2" t="b">
@@ -2379,7 +2444,7 @@
       </c>
     </row>
     <row r="157" spans="1:6">
-      <c r="A157" s="1">
+      <c r="A157" s="5">
         <v>156</v>
       </c>
       <c r="E157" s="2" t="b">
@@ -2390,7 +2455,7 @@
       </c>
     </row>
     <row r="158" spans="1:6">
-      <c r="A158" s="1">
+      <c r="A158" s="5">
         <v>157</v>
       </c>
       <c r="E158" s="2" t="b">
@@ -2401,7 +2466,7 @@
       </c>
     </row>
     <row r="159" spans="1:6">
-      <c r="A159" s="1">
+      <c r="A159" s="5">
         <v>158</v>
       </c>
       <c r="E159" s="2" t="b">
@@ -2412,7 +2477,7 @@
       </c>
     </row>
     <row r="160" spans="1:6">
-      <c r="A160" s="1">
+      <c r="A160" s="5">
         <v>159</v>
       </c>
       <c r="E160" s="2" t="b">
@@ -2423,7 +2488,7 @@
       </c>
     </row>
     <row r="161" spans="1:6">
-      <c r="A161" s="1">
+      <c r="A161" s="5">
         <v>160</v>
       </c>
       <c r="E161" s="2" t="b">
@@ -2434,7 +2499,7 @@
       </c>
     </row>
     <row r="162" spans="1:6">
-      <c r="A162" s="1">
+      <c r="A162" s="5">
         <v>161</v>
       </c>
       <c r="E162" s="2" t="b">
@@ -2445,7 +2510,7 @@
       </c>
     </row>
     <row r="163" spans="1:6">
-      <c r="A163" s="1">
+      <c r="A163" s="5">
         <v>162</v>
       </c>
       <c r="E163" s="2" t="b">
@@ -2456,7 +2521,7 @@
       </c>
     </row>
     <row r="164" spans="1:6">
-      <c r="A164" s="1">
+      <c r="A164" s="5">
         <v>163</v>
       </c>
       <c r="E164" s="2" t="b">
@@ -2467,7 +2532,7 @@
       </c>
     </row>
     <row r="165" spans="1:6">
-      <c r="A165" s="1">
+      <c r="A165" s="5">
         <v>164</v>
       </c>
       <c r="E165" s="2" t="b">
@@ -2478,7 +2543,7 @@
       </c>
     </row>
     <row r="166" spans="1:6">
-      <c r="A166" s="1">
+      <c r="A166" s="5">
         <v>165</v>
       </c>
       <c r="E166" s="2" t="b">
@@ -2489,7 +2554,7 @@
       </c>
     </row>
     <row r="167" spans="1:6">
-      <c r="A167" s="1">
+      <c r="A167" s="5">
         <v>166</v>
       </c>
       <c r="E167" s="2" t="b">
@@ -2500,7 +2565,7 @@
       </c>
     </row>
     <row r="168" spans="1:6">
-      <c r="A168" s="1">
+      <c r="A168" s="5">
         <v>167</v>
       </c>
       <c r="E168" s="2" t="b">
@@ -2511,7 +2576,7 @@
       </c>
     </row>
     <row r="169" spans="1:6">
-      <c r="A169" s="1">
+      <c r="A169" s="5">
         <v>168</v>
       </c>
       <c r="E169" s="2" t="b">
@@ -2522,7 +2587,7 @@
       </c>
     </row>
     <row r="170" spans="1:6">
-      <c r="A170" s="1">
+      <c r="A170" s="5">
         <v>169</v>
       </c>
       <c r="E170" s="2" t="b">

</xml_diff>

<commit_message>
Ajout corrigés: EX-CH01-001 et EX-CH01-002
</commit_message>
<xml_diff>
--- a/AVANCEMENT.xlsx
+++ b/AVANCEMENT.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/noemiejordi/Documents/_Ecole/03-Cycle3/MAT/01-Sequences/VLM/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E891258-1D1D-D14F-A6E5-9B3DB2404584}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53A40394-687E-F143-B7E4-BB1208AE6A0D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-5080" yWindow="-21000" windowWidth="38400" windowHeight="21000" xr2:uid="{3DF85CC0-EEB2-D042-841B-46056AFB3A80}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="33">
   <si>
     <t>ex-008</t>
   </si>
@@ -557,7 +557,7 @@
     <col min="4" max="4" width="12.83203125" style="1" customWidth="1"/>
     <col min="5" max="6" width="14.6640625" style="1" customWidth="1"/>
     <col min="7" max="7" width="54.1640625" style="1" customWidth="1"/>
-    <col min="8" max="8" width="10.83203125" style="1"/>
+    <col min="8" max="8" width="10.83203125" style="5"/>
     <col min="9" max="12" width="16" style="1" customWidth="1"/>
     <col min="13" max="13" width="54.1640625" style="1" customWidth="1"/>
     <col min="14" max="16384" width="10.83203125" style="1"/>
@@ -585,7 +585,7 @@
       <c r="G1" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="H1" s="4" t="s">
         <v>32</v>
       </c>
       <c r="I1" s="3" t="s">
@@ -628,7 +628,7 @@
         <v>1</v>
       </c>
       <c r="K2" s="2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L2" s="2" t="b">
         <v>0</v>
@@ -681,10 +681,10 @@
         <v>1</v>
       </c>
       <c r="F4" s="2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H4" s="5">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="I4" s="1" t="s">
         <v>31</v>
@@ -718,6 +718,18 @@
       <c r="F5" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="H5" s="5">
+        <v>17</v>
+      </c>
+      <c r="J5" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="K5" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="L5" s="2" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="6" spans="1:13">
       <c r="A6" s="5">
@@ -736,6 +748,18 @@
         <v>1</v>
       </c>
       <c r="F6" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H6" s="5">
+        <v>18</v>
+      </c>
+      <c r="J6" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="K6" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="L6" s="2" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Ajout exercice EX-CH02-012 : vecteurs colinéaires
</commit_message>
<xml_diff>
--- a/AVANCEMENT.xlsx
+++ b/AVANCEMENT.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10802"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10810"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/noemiejordi/Documents/_Ecole/03-Cycle3/MAT/01-Sequences/VLM/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53A40394-687E-F143-B7E4-BB1208AE6A0D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DDEA73B9-AF77-C84B-8031-8E4692886FAB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-5080" yWindow="-21000" windowWidth="38400" windowHeight="21000" xr2:uid="{3DF85CC0-EEB2-D042-841B-46056AFB3A80}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" xr2:uid="{3DF85CC0-EEB2-D042-841B-46056AFB3A80}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -716,7 +716,7 @@
         <v>1</v>
       </c>
       <c r="F5" s="2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H5" s="5">
         <v>17</v>
@@ -748,7 +748,7 @@
         <v>1</v>
       </c>
       <c r="F6" s="2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H6" s="5">
         <v>18</v>
@@ -780,7 +780,7 @@
         <v>1</v>
       </c>
       <c r="F7" s="2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8" spans="1:13">
@@ -800,7 +800,7 @@
         <v>1</v>
       </c>
       <c r="F8" s="2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -820,7 +820,7 @@
         <v>1</v>
       </c>
       <c r="F9" s="2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -840,7 +840,7 @@
         <v>1</v>
       </c>
       <c r="F10" s="2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11" spans="1:13">

</xml_diff>